<commit_message>
Completed team status report 20261005
</commit_message>
<xml_diff>
--- a/Team-StatusReport.xlsx
+++ b/Team-StatusReport.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rjones\Documents\C67\Team Status Reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vanan\Repositories\mthree-project-team-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D0FB31-DB1A-4E5E-9409-0655FFDAFAFD}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D11C81D-9B07-4E07-A778-C2FD7A3F3614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="10" windowWidth="16760" windowHeight="10790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Status Report" sheetId="1" r:id="rId1"/>
+    <sheet name="Status Report Template" sheetId="1" r:id="rId1"/>
+    <sheet name="261005-StatusReport" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="53">
   <si>
     <t>Project</t>
   </si>
@@ -147,7 +148,100 @@
     <t>Comment/Status %</t>
   </si>
   <si>
-    <t>Status Report for Team #</t>
+    <t>Status Report for Team 1</t>
+  </si>
+  <si>
+    <t>Vrishti</t>
+  </si>
+  <si>
+    <t>Team effort</t>
+  </si>
+  <si>
+    <t>Setup a Scrum Board on GitHub</t>
+  </si>
+  <si>
+    <t>Security &amp; User Setup</t>
+  </si>
+  <si>
+    <t>Saif - Okay</t>
+  </si>
+  <si>
+    <t>Client Goals</t>
+  </si>
+  <si>
+    <t>Favour - Okay</t>
+  </si>
+  <si>
+    <t>Planned Class Diagram</t>
+  </si>
+  <si>
+    <t>Planned ERD</t>
+  </si>
+  <si>
+    <t>Planned User Stories</t>
+  </si>
+  <si>
+    <t>API Setup &amp; Food Lookup</t>
+  </si>
+  <si>
+    <t>Consultant Clients</t>
+  </si>
+  <si>
+    <t>Food Diary Entries</t>
+  </si>
+  <si>
+    <t>Tracking Goals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daily Diary Feedback </t>
+  </si>
+  <si>
+    <t>Stretch</t>
+  </si>
+  <si>
+    <t>Food Recommendations</t>
+  </si>
+  <si>
+    <t>User Management Plus</t>
+  </si>
+  <si>
+    <t>Client Recipies</t>
+  </si>
+  <si>
+    <t>v2.0</t>
+  </si>
+  <si>
+    <t>Recipe Recommendations</t>
+  </si>
+  <si>
+    <t>via mthree email/teams</t>
+  </si>
+  <si>
+    <t>Presentation Preparation</t>
+  </si>
+  <si>
+    <t>Date Completed</t>
+  </si>
+  <si>
+    <t>Allowing team to split-up and start working on tasks today</t>
+  </si>
+  <si>
+    <t>Initial Project Setup on GitHub</t>
+  </si>
+  <si>
+    <t>Vrishti - Okay. Best to set-up for security now to avoid potential issues later</t>
+  </si>
+  <si>
+    <t>We've mostly planned our user stories, class diagram and ERD last week. User stories have also been grouped into work packages and organised on a scrum board on GitHub. And, we're ready to start development today.</t>
+  </si>
+  <si>
+    <t>[As listed in issues/tasks on GitHub]</t>
+  </si>
+  <si>
+    <t>Testing as we go through features</t>
+  </si>
+  <si>
+    <t>Comment</t>
   </si>
 </sst>
 </file>
@@ -157,7 +251,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color indexed="8"/>
@@ -214,8 +308,34 @@
       <color indexed="17"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -256,6 +376,12 @@
       <patternFill patternType="solid">
         <fgColor indexed="19"/>
         <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -478,9 +604,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="90">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -493,16 +619,16 @@
     <xf numFmtId="49" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -592,61 +718,61 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -672,6 +798,78 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="16" fontId="8" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1864,15 +2062,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G35"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="6" width="15.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="45.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="6" width="15.6875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="45.3125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.8125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.8125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="58" t="s">
         <v>21</v>
       </c>
@@ -1883,7 +2081,7 @@
       <c r="F1" s="59"/>
       <c r="G1" s="60"/>
     </row>
-    <row r="2" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="2"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -1892,7 +2090,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="4"/>
     </row>
-    <row r="3" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="5" t="s">
         <v>0</v>
       </c>
@@ -1905,7 +2103,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="9"/>
     </row>
-    <row r="4" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
@@ -1920,7 +2118,7 @@
       <c r="F4" s="14"/>
       <c r="G4" s="15"/>
     </row>
-    <row r="5" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="10" t="s">
         <v>5</v>
       </c>
@@ -1933,7 +2131,7 @@
       <c r="F5" s="62"/>
       <c r="G5" s="63"/>
     </row>
-    <row r="6" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="10" t="s">
         <v>7</v>
       </c>
@@ -1944,7 +2142,7 @@
       <c r="F6" s="64"/>
       <c r="G6" s="65"/>
     </row>
-    <row r="7" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7" s="18"/>
       <c r="B7" s="19"/>
       <c r="C7" s="7"/>
@@ -1953,7 +2151,7 @@
       <c r="F7" s="21"/>
       <c r="G7" s="22"/>
     </row>
-    <row r="8" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
@@ -1964,7 +2162,7 @@
       <c r="F8" s="6"/>
       <c r="G8" s="9"/>
     </row>
-    <row r="9" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="23" t="s">
         <v>9</v>
       </c>
@@ -1975,7 +2173,7 @@
       <c r="F9" s="24"/>
       <c r="G9" s="25"/>
     </row>
-    <row r="10" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A10" s="26" t="s">
         <v>18</v>
       </c>
@@ -1988,7 +2186,7 @@
       <c r="F10" s="14"/>
       <c r="G10" s="15"/>
     </row>
-    <row r="11" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="28"/>
       <c r="B11" s="16"/>
       <c r="C11" s="29"/>
@@ -1997,7 +2195,7 @@
       <c r="F11" s="29"/>
       <c r="G11" s="30"/>
     </row>
-    <row r="12" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="28"/>
       <c r="B12" s="16"/>
       <c r="C12" s="29"/>
@@ -2006,7 +2204,7 @@
       <c r="F12" s="29"/>
       <c r="G12" s="30"/>
     </row>
-    <row r="13" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A13" s="28"/>
       <c r="B13" s="16"/>
       <c r="C13" s="29"/>
@@ -2015,7 +2213,7 @@
       <c r="F13" s="29"/>
       <c r="G13" s="30"/>
     </row>
-    <row r="14" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A14" s="28"/>
       <c r="B14" s="16"/>
       <c r="C14" s="29"/>
@@ -2024,7 +2222,7 @@
       <c r="F14" s="29"/>
       <c r="G14" s="30"/>
     </row>
-    <row r="15" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="28"/>
       <c r="B15" s="16"/>
       <c r="C15" s="29"/>
@@ -2033,7 +2231,7 @@
       <c r="F15" s="29"/>
       <c r="G15" s="30"/>
     </row>
-    <row r="16" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A16" s="31"/>
       <c r="B16" s="19"/>
       <c r="C16" s="19"/>
@@ -2042,7 +2240,7 @@
       <c r="F16" s="19"/>
       <c r="G16" s="32"/>
     </row>
-    <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A17" s="5" t="s">
         <v>10</v>
       </c>
@@ -2059,7 +2257,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A18" s="36"/>
       <c r="B18" s="27" t="s">
         <v>14</v>
@@ -2070,7 +2268,7 @@
       <c r="F18" s="14"/>
       <c r="G18" s="15"/>
     </row>
-    <row r="19" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A19" s="37"/>
       <c r="B19" s="29"/>
       <c r="C19" s="29"/>
@@ -2079,7 +2277,7 @@
       <c r="F19" s="29"/>
       <c r="G19" s="30"/>
     </row>
-    <row r="20" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A20" s="37"/>
       <c r="B20" s="29"/>
       <c r="C20" s="29"/>
@@ -2088,7 +2286,7 @@
       <c r="F20" s="29"/>
       <c r="G20" s="30"/>
     </row>
-    <row r="21" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A21" s="37"/>
       <c r="B21" s="29"/>
       <c r="C21" s="29"/>
@@ -2097,7 +2295,7 @@
       <c r="F21" s="29"/>
       <c r="G21" s="30"/>
     </row>
-    <row r="22" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A22" s="31"/>
       <c r="B22" s="19"/>
       <c r="C22" s="19"/>
@@ -2106,7 +2304,7 @@
       <c r="F22" s="19"/>
       <c r="G22" s="32"/>
     </row>
-    <row r="23" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A23" s="5" t="s">
         <v>15</v>
       </c>
@@ -2123,7 +2321,7 @@
       </c>
       <c r="G23" s="9"/>
     </row>
-    <row r="24" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A24" s="41"/>
       <c r="B24" s="42"/>
       <c r="C24" s="42"/>
@@ -2134,7 +2332,7 @@
       <c r="F24" s="45"/>
       <c r="G24" s="46"/>
     </row>
-    <row r="25" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A25" s="47"/>
       <c r="B25" s="48"/>
       <c r="C25" s="49"/>
@@ -2145,7 +2343,7 @@
       <c r="F25" s="45"/>
       <c r="G25" s="51"/>
     </row>
-    <row r="26" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A26" s="47"/>
       <c r="B26" s="48"/>
       <c r="C26" s="49"/>
@@ -2156,7 +2354,7 @@
       <c r="F26" s="45"/>
       <c r="G26" s="51"/>
     </row>
-    <row r="27" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A27" s="47"/>
       <c r="B27" s="48"/>
       <c r="C27" s="49"/>
@@ -2167,7 +2365,7 @@
       <c r="F27" s="52"/>
       <c r="G27" s="51"/>
     </row>
-    <row r="28" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A28" s="47"/>
       <c r="B28" s="48"/>
       <c r="C28" s="49"/>
@@ -2178,7 +2376,7 @@
       <c r="F28" s="45"/>
       <c r="G28" s="51"/>
     </row>
-    <row r="29" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A29" s="47"/>
       <c r="B29" s="48"/>
       <c r="C29" s="49"/>
@@ -2189,7 +2387,7 @@
       <c r="F29" s="45"/>
       <c r="G29" s="51"/>
     </row>
-    <row r="30" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A30" s="47"/>
       <c r="B30" s="48"/>
       <c r="C30" s="49"/>
@@ -2200,7 +2398,7 @@
       <c r="F30" s="45"/>
       <c r="G30" s="51"/>
     </row>
-    <row r="31" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A31" s="47"/>
       <c r="B31" s="48"/>
       <c r="C31" s="49"/>
@@ -2211,7 +2409,7 @@
       <c r="F31" s="45"/>
       <c r="G31" s="51"/>
     </row>
-    <row r="32" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A32" s="47"/>
       <c r="B32" s="48"/>
       <c r="C32" s="49"/>
@@ -2222,7 +2420,7 @@
       <c r="F32" s="45"/>
       <c r="G32" s="51"/>
     </row>
-    <row r="33" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A33" s="47"/>
       <c r="B33" s="48"/>
       <c r="C33" s="48"/>
@@ -2233,7 +2431,7 @@
       <c r="F33" s="45"/>
       <c r="G33" s="51"/>
     </row>
-    <row r="34" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A34" s="47"/>
       <c r="B34" s="48"/>
       <c r="C34" s="48"/>
@@ -2242,7 +2440,7 @@
       <c r="F34" s="48"/>
       <c r="G34" s="51"/>
     </row>
-    <row r="35" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A35" s="55"/>
       <c r="B35" s="56"/>
       <c r="C35" s="56"/>
@@ -2250,6 +2448,555 @@
       <c r="E35" s="56"/>
       <c r="F35" s="56"/>
       <c r="G35" s="57"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="E5:G6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="1" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;"Arial,Regular"&amp;8&amp;K000000v1.0</oddHeader>
+    <oddFooter>&amp;C&amp;"Arial,Regular"&amp;8&amp;K000000
+Copyright 2018 GoLeanSixSigma.com. All Rights Reserved.</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06662D99-A88D-4421-8837-E1E94D50A084}">
+  <dimension ref="A1:G36"/>
+  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.5"/>
+  <cols>
+    <col min="1" max="1" width="15.6875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25.125" style="1" customWidth="1"/>
+    <col min="3" max="5" width="15.6875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="61.625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.8125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.8125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="58" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="60"/>
+    </row>
+    <row r="2" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="9"/>
+    </row>
+    <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A4" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="11">
+        <v>46300</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="14"/>
+      <c r="G4" s="15"/>
+    </row>
+    <row r="5" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A5" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="72" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="86" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" s="66"/>
+      <c r="G5" s="67"/>
+    </row>
+    <row r="6" spans="1:7" ht="23.65" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A6" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="73" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="69"/>
+    </row>
+    <row r="7" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A7" s="18"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="22"/>
+    </row>
+    <row r="8" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="9"/>
+    </row>
+    <row r="9" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A9" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="25"/>
+    </row>
+    <row r="10" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A10" s="75" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="76" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="77"/>
+      <c r="D10" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="77" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="15"/>
+    </row>
+    <row r="11" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A11" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="D11" s="74">
+        <v>46296</v>
+      </c>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="30"/>
+    </row>
+    <row r="12" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A12" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="29"/>
+      <c r="D12" s="74">
+        <v>46297</v>
+      </c>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="30"/>
+    </row>
+    <row r="13" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A13" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="29"/>
+      <c r="D13" s="74">
+        <v>46297</v>
+      </c>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="30"/>
+    </row>
+    <row r="14" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A14" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="29"/>
+      <c r="D14" s="74">
+        <v>46300</v>
+      </c>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="30"/>
+    </row>
+    <row r="15" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A15" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="79" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="29"/>
+      <c r="D15" s="74">
+        <v>46300</v>
+      </c>
+      <c r="E15" s="81" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" s="29"/>
+      <c r="G15" s="30"/>
+    </row>
+    <row r="16" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A16" s="31"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="32"/>
+    </row>
+    <row r="17" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="34"/>
+      <c r="D17" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A18" s="36"/>
+      <c r="B18" s="80" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="15"/>
+    </row>
+    <row r="19" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A19" s="37"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="30"/>
+    </row>
+    <row r="20" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A20" s="37"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="30"/>
+    </row>
+    <row r="21" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A21" s="37"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="30"/>
+    </row>
+    <row r="22" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A22" s="31"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="32"/>
+    </row>
+    <row r="23" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A23" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="38"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="88" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="89" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="89" t="s">
+        <v>20</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A24" s="87" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="42"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="82" t="s">
+        <v>51</v>
+      </c>
+      <c r="G24" s="48"/>
+    </row>
+    <row r="25" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A25" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" s="48"/>
+      <c r="C25" s="49"/>
+      <c r="D25" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E25" s="71">
+        <v>46301</v>
+      </c>
+      <c r="F25" s="82" t="s">
+        <v>48</v>
+      </c>
+      <c r="G25" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A26" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="48"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E26" s="71">
+        <v>46301</v>
+      </c>
+      <c r="F26" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A27" s="47" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" s="48"/>
+      <c r="C27" s="49"/>
+      <c r="D27" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E27" s="71">
+        <v>46301</v>
+      </c>
+      <c r="F27" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="G27" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A28" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" s="48"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E28" s="71">
+        <v>46301</v>
+      </c>
+      <c r="F28" s="45"/>
+      <c r="G28" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A29" s="47" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="48"/>
+      <c r="C29" s="49"/>
+      <c r="D29" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E29" s="44">
+        <v>46302</v>
+      </c>
+      <c r="F29" s="45"/>
+      <c r="G29" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A30" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="48"/>
+      <c r="C30" s="49"/>
+      <c r="D30" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E30" s="44">
+        <v>46302</v>
+      </c>
+      <c r="F30" s="45"/>
+      <c r="G30" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A31" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="48"/>
+      <c r="C31" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E31" s="44">
+        <v>46302</v>
+      </c>
+      <c r="F31" s="45"/>
+      <c r="G31" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A32" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="B32" s="48"/>
+      <c r="C32" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E32" s="44">
+        <v>46303</v>
+      </c>
+      <c r="F32" s="45"/>
+      <c r="G32" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A33" s="47" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="48"/>
+      <c r="C33" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="D33" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="E33" s="54">
+        <v>46303</v>
+      </c>
+      <c r="F33" s="45"/>
+      <c r="G33" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A34" s="83" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" s="48"/>
+      <c r="C34" s="49"/>
+      <c r="D34" s="50" t="s">
+        <v>4</v>
+      </c>
+      <c r="E34" s="44">
+        <v>46304</v>
+      </c>
+      <c r="F34" s="45"/>
+      <c r="G34" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A35" s="47" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35" s="48"/>
+      <c r="C35" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="D35" s="84"/>
+      <c r="E35" s="84"/>
+      <c r="F35" s="48"/>
+      <c r="G35" s="70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A36" s="55" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" s="56"/>
+      <c r="C36" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="D36" s="85"/>
+      <c r="E36" s="85"/>
+      <c r="F36" s="56"/>
+      <c r="G36" s="70">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Improved formatting on status report
</commit_message>
<xml_diff>
--- a/Team-StatusReport.xlsx
+++ b/Team-StatusReport.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vanan\Repositories\mthree-project-team-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D11C81D-9B07-4E07-A778-C2FD7A3F3614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A78296-928B-4F7C-A036-F2A9CE32FA83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Status Report Template" sheetId="1" r:id="rId1"/>
     <sheet name="261005-StatusReport" sheetId="4" r:id="rId2"/>
+    <sheet name="261006-StatusReport" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="62">
   <si>
     <t>Project</t>
   </si>
@@ -154,24 +155,15 @@
     <t>Vrishti</t>
   </si>
   <si>
-    <t>Team effort</t>
-  </si>
-  <si>
     <t>Setup a Scrum Board on GitHub</t>
   </si>
   <si>
     <t>Security &amp; User Setup</t>
   </si>
   <si>
-    <t>Saif - Okay</t>
-  </si>
-  <si>
     <t>Client Goals</t>
   </si>
   <si>
-    <t>Favour - Okay</t>
-  </si>
-  <si>
     <t>Planned Class Diagram</t>
   </si>
   <si>
@@ -217,9 +209,6 @@
     <t>via mthree email/teams</t>
   </si>
   <si>
-    <t>Presentation Preparation</t>
-  </si>
-  <si>
     <t>Date Completed</t>
   </si>
   <si>
@@ -238,10 +227,49 @@
     <t>[As listed in issues/tasks on GitHub]</t>
   </si>
   <si>
-    <t>Testing as we go through features</t>
-  </si>
-  <si>
     <t>Comment</t>
+  </si>
+  <si>
+    <t>Presentation Dry-Run</t>
+  </si>
+  <si>
+    <t>Presentation</t>
+  </si>
+  <si>
+    <t>Status %</t>
+  </si>
+  <si>
+    <t>(Testing as we go through features - hopefully)</t>
+  </si>
+  <si>
+    <t>Team Effort</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Saif - Okay.</t>
+  </si>
+  <si>
+    <t>Favour - Okay.</t>
+  </si>
+  <si>
+    <t>06/10/2026 1pm</t>
+  </si>
+  <si>
+    <t>07/10/2026 1pm</t>
+  </si>
+  <si>
+    <t>08/10/2026 1pm</t>
+  </si>
+  <si>
+    <t>09/10/2026 1pm</t>
+  </si>
+  <si>
+    <t>08/10/2026 3pm</t>
+  </si>
+  <si>
+    <t>Discuss deadlines</t>
   </si>
 </sst>
 </file>
@@ -330,7 +358,7 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color indexed="8"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -385,7 +413,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -600,11 +628,100 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -775,6 +892,33 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="10" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -799,78 +943,139 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="16" fontId="8" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="7" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="7" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="7" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="7" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="7" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="16" fontId="8" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2071,15 +2276,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="60"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="69"/>
     </row>
     <row r="2" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="2"/>
@@ -2127,9 +2332,9 @@
       <c r="D5" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="61"/>
-      <c r="F5" s="62"/>
-      <c r="G5" s="63"/>
+      <c r="E5" s="70"/>
+      <c r="F5" s="71"/>
+      <c r="G5" s="72"/>
     </row>
     <row r="6" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="10" t="s">
@@ -2138,9 +2343,9 @@
       <c r="B6" s="16"/>
       <c r="C6" s="7"/>
       <c r="D6" s="17"/>
-      <c r="E6" s="64"/>
-      <c r="F6" s="64"/>
-      <c r="G6" s="65"/>
+      <c r="E6" s="73"/>
+      <c r="F6" s="73"/>
+      <c r="G6" s="74"/>
     </row>
     <row r="7" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7" s="18"/>
@@ -2466,28 +2671,28 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06662D99-A88D-4421-8837-E1E94D50A084}">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="15.6875" style="1" customWidth="1"/>
     <col min="2" max="2" width="25.125" style="1" customWidth="1"/>
     <col min="3" max="5" width="15.6875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="61.625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="68.9375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9" style="1" customWidth="1"/>
     <col min="8" max="8" width="10.8125" style="1" customWidth="1"/>
     <col min="9" max="16384" width="10.8125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="60"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="69"/>
     </row>
     <row r="2" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="2"/>
@@ -2499,122 +2704,122 @@
       <c r="G2" s="4"/>
     </row>
     <row r="3" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="105" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="6"/>
+      <c r="B3" s="106"/>
       <c r="C3" s="7"/>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="105" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="9"/>
+      <c r="E3" s="107"/>
+      <c r="F3" s="107"/>
+      <c r="G3" s="106"/>
     </row>
     <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="104">
         <v>46300</v>
       </c>
       <c r="C4" s="7"/>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="95" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="14"/>
-      <c r="G4" s="15"/>
+      <c r="F4" s="96"/>
+      <c r="G4" s="97"/>
     </row>
     <row r="5" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="117" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="72" t="s">
-        <v>43</v>
+      <c r="B5" s="78" t="s">
+        <v>40</v>
       </c>
       <c r="C5" s="7"/>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="86" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5" s="66"/>
-      <c r="G5" s="67"/>
+      <c r="E5" s="81" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="82"/>
+      <c r="G5" s="82"/>
     </row>
     <row r="6" spans="1:7" ht="23.65" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="118" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="73" t="s">
+      <c r="B6" s="78" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="7"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="69"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="82"/>
+      <c r="F6" s="82"/>
+      <c r="G6" s="82"/>
     </row>
     <row r="7" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7" s="18"/>
-      <c r="B7" s="19"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="7"/>
       <c r="D7" s="20"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="22"/>
+      <c r="E7" s="79"/>
+      <c r="F7" s="79"/>
+      <c r="G7" s="80"/>
     </row>
     <row r="8" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="105" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="9"/>
+      <c r="B8" s="107"/>
+      <c r="C8" s="107"/>
+      <c r="D8" s="107"/>
+      <c r="E8" s="107"/>
+      <c r="F8" s="107"/>
+      <c r="G8" s="106"/>
     </row>
     <row r="9" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="87" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="25"/>
+      <c r="B9" s="115"/>
+      <c r="C9" s="115"/>
+      <c r="D9" s="115"/>
+      <c r="E9" s="115"/>
+      <c r="F9" s="115"/>
+      <c r="G9" s="116"/>
     </row>
     <row r="10" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A10" s="75" t="s">
+      <c r="A10" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="76" t="s">
+      <c r="B10" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="77"/>
-      <c r="D10" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="77" t="s">
-        <v>52</v>
+      <c r="C10" s="60"/>
+      <c r="D10" s="76" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="60" t="s">
+        <v>47</v>
       </c>
       <c r="F10" s="14"/>
       <c r="G10" s="15"/>
     </row>
     <row r="11" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="28" t="s">
-        <v>23</v>
+      <c r="A11" s="61" t="s">
+        <v>52</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C11" s="29"/>
-      <c r="D11" s="74">
+      <c r="D11" s="77">
         <v>46296</v>
       </c>
       <c r="E11" s="29"/>
@@ -2622,14 +2827,14 @@
       <c r="G11" s="30"/>
     </row>
     <row r="12" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A12" s="28" t="s">
-        <v>23</v>
+      <c r="A12" s="61" t="s">
+        <v>52</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C12" s="29"/>
-      <c r="D12" s="74">
+      <c r="D12" s="77">
         <v>46297</v>
       </c>
       <c r="E12" s="29"/>
@@ -2637,14 +2842,14 @@
       <c r="G12" s="30"/>
     </row>
     <row r="13" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A13" s="28" t="s">
-        <v>23</v>
+      <c r="A13" s="61" t="s">
+        <v>52</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C13" s="29"/>
-      <c r="D13" s="74">
+      <c r="D13" s="77">
         <v>46297</v>
       </c>
       <c r="E13" s="29"/>
@@ -2652,14 +2857,14 @@
       <c r="G13" s="30"/>
     </row>
     <row r="14" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A14" s="78" t="s">
+      <c r="A14" s="61" t="s">
         <v>22</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C14" s="29"/>
-      <c r="D14" s="74">
+      <c r="D14" s="77">
         <v>46300</v>
       </c>
       <c r="E14" s="29"/>
@@ -2667,18 +2872,18 @@
       <c r="G14" s="30"/>
     </row>
     <row r="15" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A15" s="78" t="s">
+      <c r="A15" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="79" t="s">
-        <v>47</v>
+      <c r="B15" s="62" t="s">
+        <v>43</v>
       </c>
       <c r="C15" s="29"/>
-      <c r="D15" s="74">
+      <c r="D15" s="77">
         <v>46300</v>
       </c>
-      <c r="E15" s="81" t="s">
-        <v>46</v>
+      <c r="E15" s="64" t="s">
+        <v>42</v>
       </c>
       <c r="F15" s="29"/>
       <c r="G15" s="30"/>
@@ -2693,25 +2898,25 @@
       <c r="G16" s="32"/>
     </row>
     <row r="17" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="105" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="34"/>
-      <c r="D17" s="33" t="s">
+      <c r="C17" s="109"/>
+      <c r="D17" s="108" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="35" t="s">
+      <c r="E17" s="109"/>
+      <c r="F17" s="109"/>
+      <c r="G17" s="110" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A18" s="36"/>
-      <c r="B18" s="80" t="s">
+      <c r="B18" s="63" t="s">
         <v>14</v>
       </c>
       <c r="C18" s="14"/>
@@ -2757,251 +2962,811 @@
       <c r="G22" s="32"/>
     </row>
     <row r="23" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="105" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="38"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="88" t="s">
+      <c r="B23" s="111"/>
+      <c r="C23" s="112" t="s">
+        <v>53</v>
+      </c>
+      <c r="D23" s="113" t="s">
         <v>16</v>
       </c>
-      <c r="E23" s="89" t="s">
+      <c r="E23" s="113" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="89" t="s">
-        <v>20</v>
-      </c>
-      <c r="G23" s="9"/>
+      <c r="F23" s="113" t="s">
+        <v>47</v>
+      </c>
+      <c r="G23" s="114" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="24" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A24" s="87" t="s">
-        <v>50</v>
-      </c>
-      <c r="B24" s="42"/>
-      <c r="C24" s="49"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="44"/>
-      <c r="F24" s="82" t="s">
+      <c r="A24" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="102"/>
+      <c r="C24" s="103"/>
+      <c r="D24" s="88"/>
+      <c r="E24" s="88"/>
+      <c r="F24" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="G24" s="48"/>
+      <c r="G24" s="88"/>
     </row>
     <row r="25" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A25" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25" s="48"/>
-      <c r="C25" s="49"/>
-      <c r="D25" s="50" t="s">
+      <c r="A25" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="42"/>
+      <c r="C25" s="92"/>
+      <c r="D25" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="71">
-        <v>46301</v>
-      </c>
-      <c r="F25" s="82" t="s">
-        <v>48</v>
-      </c>
-      <c r="G25" s="70">
-        <v>0</v>
+      <c r="E25" s="99" t="s">
+        <v>56</v>
+      </c>
+      <c r="F25" s="90" t="s">
+        <v>44</v>
+      </c>
+      <c r="G25" s="91">
+        <v>0.1</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A26" s="47" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B26" s="48"/>
-      <c r="C26" s="49"/>
-      <c r="D26" s="50" t="s">
+      <c r="C26" s="92"/>
+      <c r="D26" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="E26" s="71">
-        <v>46301</v>
-      </c>
-      <c r="F26" s="45" t="s">
-        <v>26</v>
-      </c>
-      <c r="G26" s="70">
+      <c r="E26" s="100" t="s">
+        <v>56</v>
+      </c>
+      <c r="F26" s="90" t="s">
+        <v>54</v>
+      </c>
+      <c r="G26" s="91">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A27" s="47" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B27" s="48"/>
-      <c r="C27" s="49"/>
-      <c r="D27" s="50" t="s">
+      <c r="C27" s="92"/>
+      <c r="D27" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="71">
-        <v>46301</v>
-      </c>
-      <c r="F27" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="G27" s="70">
-        <v>0</v>
+      <c r="E27" s="100" t="s">
+        <v>56</v>
+      </c>
+      <c r="F27" s="98" t="s">
+        <v>55</v>
+      </c>
+      <c r="G27" s="91">
+        <v>0.1</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A28" s="47" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B28" s="48"/>
-      <c r="C28" s="49"/>
-      <c r="D28" s="50" t="s">
+      <c r="C28" s="92"/>
+      <c r="D28" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="71">
-        <v>46301</v>
-      </c>
-      <c r="F28" s="45"/>
-      <c r="G28" s="70">
-        <v>0</v>
+      <c r="E28" s="100" t="s">
+        <v>56</v>
+      </c>
+      <c r="F28" s="91"/>
+      <c r="G28" s="91">
+        <v>0.1</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A29" s="47" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B29" s="48"/>
-      <c r="C29" s="49"/>
-      <c r="D29" s="50" t="s">
+      <c r="C29" s="92"/>
+      <c r="D29" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="44">
-        <v>46302</v>
-      </c>
-      <c r="F29" s="45"/>
-      <c r="G29" s="70">
+      <c r="E29" s="100" t="s">
+        <v>57</v>
+      </c>
+      <c r="F29" s="91"/>
+      <c r="G29" s="91">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A30" s="47" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B30" s="48"/>
-      <c r="C30" s="49"/>
-      <c r="D30" s="50" t="s">
+      <c r="C30" s="92"/>
+      <c r="D30" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="44">
-        <v>46302</v>
-      </c>
-      <c r="F30" s="45"/>
-      <c r="G30" s="70">
+      <c r="E30" s="100" t="s">
+        <v>57</v>
+      </c>
+      <c r="F30" s="91"/>
+      <c r="G30" s="91">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A31" s="47" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B31" s="48"/>
-      <c r="C31" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="D31" s="50" t="s">
+      <c r="C31" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="D31" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="44">
-        <v>46302</v>
-      </c>
-      <c r="F31" s="45"/>
-      <c r="G31" s="70">
+      <c r="E31" s="100" t="s">
+        <v>57</v>
+      </c>
+      <c r="F31" s="91"/>
+      <c r="G31" s="91">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A32" s="47" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B32" s="48"/>
-      <c r="C32" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="D32" s="50" t="s">
+      <c r="C32" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="E32" s="44">
-        <v>46303</v>
-      </c>
-      <c r="F32" s="45"/>
-      <c r="G32" s="70">
+      <c r="E32" s="100" t="s">
+        <v>58</v>
+      </c>
+      <c r="F32" s="91"/>
+      <c r="G32" s="91">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A33" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="B33" s="48"/>
+      <c r="C33" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="D33" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E33" s="100" t="s">
+        <v>58</v>
+      </c>
+      <c r="F33" s="91"/>
+      <c r="G33" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A34" s="75" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="48"/>
+      <c r="C34" s="92"/>
+      <c r="D34" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E34" s="100" t="s">
+        <v>60</v>
+      </c>
+      <c r="F34" s="90"/>
+      <c r="G34" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A35" s="75" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="48"/>
+      <c r="C35" s="92"/>
+      <c r="D35" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E35" s="100" t="s">
+        <v>59</v>
+      </c>
+      <c r="F35" s="91"/>
+      <c r="G35" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A36" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36" s="48"/>
+      <c r="C36" s="92" t="s">
+        <v>38</v>
+      </c>
+      <c r="D36" s="89"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="92"/>
+      <c r="G36" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A37" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="B33" s="48"/>
-      <c r="C33" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="D33" s="53" t="s">
-        <v>4</v>
-      </c>
-      <c r="E33" s="54">
-        <v>46303</v>
-      </c>
-      <c r="F33" s="45"/>
-      <c r="G33" s="70">
+      <c r="B37" s="56"/>
+      <c r="C37" s="93" t="s">
+        <v>38</v>
+      </c>
+      <c r="D37" s="66"/>
+      <c r="E37" s="66"/>
+      <c r="F37" s="93"/>
+      <c r="G37" s="91">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A34" s="83" t="s">
-        <v>44</v>
-      </c>
-      <c r="B34" s="48"/>
-      <c r="C34" s="49"/>
-      <c r="D34" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="E34" s="44">
-        <v>46304</v>
-      </c>
-      <c r="F34" s="45"/>
-      <c r="G34" s="70">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A35" s="47" t="s">
-        <v>40</v>
-      </c>
-      <c r="B35" s="48"/>
-      <c r="C35" s="48" t="s">
-        <v>41</v>
-      </c>
-      <c r="D35" s="84"/>
-      <c r="E35" s="84"/>
-      <c r="F35" s="48"/>
-      <c r="G35" s="70">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A36" s="55" t="s">
-        <v>42</v>
-      </c>
-      <c r="B36" s="56"/>
-      <c r="C36" s="56" t="s">
-        <v>41</v>
-      </c>
-      <c r="D36" s="85"/>
-      <c r="E36" s="85"/>
-      <c r="F36" s="56"/>
-      <c r="G36" s="70">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="5">
+    <mergeCell ref="A24:C24"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="E5:G6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E4:G4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="1" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;"Arial,Regular"&amp;8&amp;K000000v1.0</oddHeader>
+    <oddFooter>&amp;C&amp;"Arial,Regular"&amp;8&amp;K000000
+Copyright 2018 GoLeanSixSigma.com. All Rights Reserved.</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4701350D-318D-4CD0-A500-65EB319D1675}">
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.5"/>
+  <cols>
+    <col min="1" max="1" width="15.6875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25.125" style="1" customWidth="1"/>
+    <col min="3" max="5" width="15.6875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="68.9375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.8125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.8125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="67" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="69"/>
+    </row>
+    <row r="2" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A3" s="105" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="106"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="105" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="107"/>
+      <c r="F3" s="107"/>
+      <c r="G3" s="106"/>
+    </row>
+    <row r="4" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A4" s="83" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="104">
+        <v>46301</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="86" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="95" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="96"/>
+      <c r="G4" s="97"/>
+    </row>
+    <row r="5" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A5" s="117" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="78" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="84" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="81"/>
+      <c r="F5" s="82"/>
+      <c r="G5" s="82"/>
+    </row>
+    <row r="6" spans="1:7" ht="23.65" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A6" s="118" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="78"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="82"/>
+      <c r="F6" s="82"/>
+      <c r="G6" s="82"/>
+    </row>
+    <row r="7" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A7" s="18"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="79"/>
+      <c r="F7" s="79"/>
+      <c r="G7" s="80"/>
+    </row>
+    <row r="8" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A8" s="105" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="107"/>
+      <c r="C8" s="107"/>
+      <c r="D8" s="107"/>
+      <c r="E8" s="107"/>
+      <c r="F8" s="107"/>
+      <c r="G8" s="106"/>
+    </row>
+    <row r="9" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A9" s="87" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="115"/>
+      <c r="C9" s="115"/>
+      <c r="D9" s="115"/>
+      <c r="E9" s="115"/>
+      <c r="F9" s="115"/>
+      <c r="G9" s="116"/>
+    </row>
+    <row r="10" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A10" s="58" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="59" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="60"/>
+      <c r="D10" s="76" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="15"/>
+    </row>
+    <row r="11" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A11" s="61"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="77"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="30"/>
+    </row>
+    <row r="12" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A12" s="61"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="77"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="30"/>
+    </row>
+    <row r="13" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A13" s="61"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="30"/>
+    </row>
+    <row r="14" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A14" s="61"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="30"/>
+    </row>
+    <row r="15" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A15" s="61"/>
+      <c r="B15" s="62"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="77"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="30"/>
+    </row>
+    <row r="16" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A16" s="31"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="32"/>
+    </row>
+    <row r="17" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A17" s="105" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="108" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="109"/>
+      <c r="D17" s="108" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="109"/>
+      <c r="F17" s="109"/>
+      <c r="G17" s="110" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A18" s="36"/>
+      <c r="B18" s="63" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="15"/>
+    </row>
+    <row r="19" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A19" s="37"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="30"/>
+    </row>
+    <row r="20" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A20" s="37"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="30"/>
+    </row>
+    <row r="21" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A21" s="37"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="30"/>
+    </row>
+    <row r="22" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A22" s="31"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="32"/>
+    </row>
+    <row r="23" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A23" s="105" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="111"/>
+      <c r="C23" s="112" t="s">
+        <v>53</v>
+      </c>
+      <c r="D23" s="113" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="113" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="113" t="s">
+        <v>47</v>
+      </c>
+      <c r="G23" s="114" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A24" s="101" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="102"/>
+      <c r="C24" s="103"/>
+      <c r="D24" s="88"/>
+      <c r="E24" s="88"/>
+      <c r="F24" s="88" t="s">
+        <v>51</v>
+      </c>
+      <c r="G24" s="88"/>
+    </row>
+    <row r="25" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A25" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="42"/>
+      <c r="C25" s="92"/>
+      <c r="D25" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E25" s="99" t="s">
+        <v>56</v>
+      </c>
+      <c r="F25" s="90"/>
+      <c r="G25" s="91">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A26" s="47" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="48"/>
+      <c r="C26" s="92"/>
+      <c r="D26" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E26" s="100" t="s">
+        <v>56</v>
+      </c>
+      <c r="F26" s="90"/>
+      <c r="G26" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A27" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="48"/>
+      <c r="C27" s="92"/>
+      <c r="D27" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E27" s="100" t="s">
+        <v>56</v>
+      </c>
+      <c r="F27" s="98"/>
+      <c r="G27" s="91">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A28" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="48"/>
+      <c r="C28" s="92"/>
+      <c r="D28" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E28" s="100" t="s">
+        <v>56</v>
+      </c>
+      <c r="F28" s="91"/>
+      <c r="G28" s="91">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A29" s="47" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="48"/>
+      <c r="C29" s="92"/>
+      <c r="D29" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E29" s="100" t="s">
+        <v>57</v>
+      </c>
+      <c r="F29" s="91"/>
+      <c r="G29" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A30" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="48"/>
+      <c r="C30" s="92"/>
+      <c r="D30" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E30" s="100" t="s">
+        <v>57</v>
+      </c>
+      <c r="F30" s="91"/>
+      <c r="G30" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A31" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="48"/>
+      <c r="C31" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="D31" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E31" s="100" t="s">
+        <v>57</v>
+      </c>
+      <c r="F31" s="91"/>
+      <c r="G31" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A32" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" s="48"/>
+      <c r="C32" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E32" s="100" t="s">
+        <v>58</v>
+      </c>
+      <c r="F32" s="91"/>
+      <c r="G32" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A33" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="B33" s="48"/>
+      <c r="C33" s="92" t="s">
+        <v>34</v>
+      </c>
+      <c r="D33" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E33" s="100" t="s">
+        <v>58</v>
+      </c>
+      <c r="F33" s="91"/>
+      <c r="G33" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A34" s="75" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="48"/>
+      <c r="C34" s="92"/>
+      <c r="D34" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E34" s="100" t="s">
+        <v>60</v>
+      </c>
+      <c r="F34" s="90"/>
+      <c r="G34" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A35" s="75" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="48"/>
+      <c r="C35" s="92"/>
+      <c r="D35" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="E35" s="100" t="s">
+        <v>59</v>
+      </c>
+      <c r="F35" s="91"/>
+      <c r="G35" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A36" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36" s="48"/>
+      <c r="C36" s="92" t="s">
+        <v>38</v>
+      </c>
+      <c r="D36" s="89"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="92"/>
+      <c r="G36" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="16.05" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A37" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="56"/>
+      <c r="C37" s="93" t="s">
+        <v>38</v>
+      </c>
+      <c r="D37" s="66"/>
+      <c r="E37" s="66"/>
+      <c r="F37" s="93"/>
+      <c r="G37" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="E39" s="119" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:G6"/>
+    <mergeCell ref="A24:C24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="1" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>

</xml_diff>